<commit_message>
Correct 07 risk register: fix duplicated summary review-date sentence; reword R-02 mitigation to fit reusable Stripe Payment Links
</commit_message>
<xml_diff>
--- a/07-risk-register/07-risk-register-lab.xlsx
+++ b/07-risk-register/07-risk-register-lab.xlsx
@@ -301,7 +301,7 @@
     <t>Stripe payment links are leaked or misused (card testing, fake links sent to clients), causing chargebacks, fees, and possible Stripe account suspension.</t>
   </si>
   <si>
-    <t>Use one-time Stripe invoices instead of reusable links; deactivate links after payment; keep Stripe Radar fraud screening on; enforce MFA on the Stripe dashboard; tell clients how real invoices arrive.</t>
+    <t>Keep Stripe Radar fraud screening on; enforce MFA on the Stripe dashboard; validate webhook signatures and charged amounts against the catalog; store the Stripe secret key in AWS SSM Parameter Store (not in code); deactivate only genuinely one-off links after use; tell clients how legitimate payment links are shared.</t>
   </si>
   <si>
     <t>Business Owner</t>
@@ -437,7 +437,7 @@
   </si>
   <si>
     <t>This register identifies 12 risks across security, vendor, and business categories. Before mitigation, four risks scored High. The top five are: compromised AWS root or admin credentials (R-01, score 20), Stripe payment link misuse (R-02, 16), phishing that steals a team login (R-05, 16), dependence on a single person for platform knowledge and admin access (R-08, 16), and loss of client files without a working backup (R-04, 12). These matter because each could stop payments, expose the AWS account, or lose client work, which would directly hurt revenue and reputation for a small media studio.
-The Business Owner owns four of the top five risks; the ISSM owns R-01. Key mitigations are MFA on all accounts, removing root access keys and using least-privilege IAM roles, one-time Stripe invoices with fraud screening, documented runbooks with a second trusted admin, and tested 3-2-1 backups. After mitigation, every risk drops to Low except R-01, which remains Medium (residual 10) because the impact of a full account takeover stays severe. R-01 should stay a leadership priority. The next review is 2026-11-12 for the High-rated risks, with R-01 reviewed by 2026-11-12 for the High-rated risks, with R-01 reviewed by 2026-11-15.</t>
+The Business Owner owns four of the top five risks; the ISSM owns R-01. Key mitigations are MFA on all accounts, removing root access keys and using least-privilege IAM roles, one-time Stripe invoices with fraud screening, documented runbooks with a second trusted admin, and tested 3-2-1 backups. After mitigation, every risk drops to Low except R-01, which remains Medium (residual 10) because the impact of a full account takeover stays severe. R-01 should stay a leadership priority. The next review is 2026-11-12 (R-02), with R-01 reviewed by 2026-11-15 and the remaining High-rated risks by 2026-12-12.</t>
   </si>
 </sst>
 </file>

</xml_diff>